<commit_message>
Refresh Intercom directory from 15-Sep Excel and regenerate Contact Center template.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/templates/SNHC_Intercom_Directory_Template.xlsx
+++ b/public/templates/SNHC_Intercom_Directory_Template.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intercom Directory" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Intercom Directory'!$A$1:$I$143</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Intercom Directory'!$A$1:$I$152</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -593,14 +593,14 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Pre-filled rows: 142 contacts from SNHC Extension Directory (as on 05-Sep-2026).</t>
+          <t>Pre-filled rows: 151 contacts from SNHC Extension Directory (as on 15-Sep-2026).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Blank cells are intentional — please update and return to IT / Admin.</t>
+          <t>Blank Section / Floor / Mobile / Email — please fill location details and return to IT / Admin.</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I143"/>
+  <dimension ref="A1:I152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -744,7 +744,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Ajay Jangra</t>
+          <t>Aman -HR</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -754,14 +754,14 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>BME</t>
+          <t>Aman -HR</t>
         </is>
       </c>
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="4" t="n"/>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>1545</t>
+          <t>1588</t>
         </is>
       </c>
       <c r="G4" s="4" t="n"/>
@@ -775,7 +775,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Vishal Rana</t>
+          <t>Anoop Store</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -785,14 +785,14 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>BME</t>
+          <t>Anoop Store</t>
         </is>
       </c>
       <c r="D5" s="4" t="n"/>
       <c r="E5" s="4" t="n"/>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>1546</t>
+          <t>1540</t>
         </is>
       </c>
       <c r="G5" s="4" t="n"/>
@@ -806,7 +806,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Blood Bank- Reception</t>
+          <t>Ajay Jangra</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -816,14 +816,14 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Blood Bank- Reception</t>
+          <t>BME</t>
         </is>
       </c>
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>1202</t>
+          <t>1545</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -837,7 +837,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Cemo-Office</t>
+          <t>Vishal Rana</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -847,14 +847,14 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Cemo-Office</t>
+          <t>BME</t>
         </is>
       </c>
       <c r="D7" s="4" t="n"/>
       <c r="E7" s="4" t="n"/>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>1222</t>
+          <t>1546</t>
         </is>
       </c>
       <c r="G7" s="4" t="n"/>
@@ -868,7 +868,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Chemotherapy NS-1</t>
+          <t>Blood Bank- Reception</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -878,14 +878,14 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Chemotherapy NS-1</t>
+          <t>Blood Bank- Reception</t>
         </is>
       </c>
       <c r="D8" s="4" t="n"/>
       <c r="E8" s="4" t="n"/>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>1280</t>
+          <t>1202</t>
         </is>
       </c>
       <c r="G8" s="4" t="n"/>
@@ -899,7 +899,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Chemotherapy NS-1</t>
+          <t>Cemo-Office</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -909,14 +909,14 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Chemotherapy NS-1</t>
+          <t>Cemo-Office</t>
         </is>
       </c>
       <c r="D9" s="4" t="n"/>
       <c r="E9" s="4" t="n"/>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>1281</t>
+          <t>1222</t>
         </is>
       </c>
       <c r="G9" s="4" t="n"/>
@@ -930,7 +930,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Chemotherapy NS-2</t>
+          <t>Chemotherapy NS-1</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -940,14 +940,14 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Chemotherapy NS-2</t>
+          <t>Chemotherapy NS-1</t>
         </is>
       </c>
       <c r="D10" s="4" t="n"/>
       <c r="E10" s="4" t="n"/>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>1282</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="G10" s="4" t="n"/>
@@ -961,7 +961,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Chemotherapy- Doctor Room</t>
+          <t>Chemotherapy NS-1</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -971,14 +971,14 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Chemotherapy- Doctor Room</t>
+          <t>Chemotherapy NS-1</t>
         </is>
       </c>
       <c r="D11" s="4" t="n"/>
       <c r="E11" s="4" t="n"/>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>1270</t>
+          <t>1281</t>
         </is>
       </c>
       <c r="G11" s="4" t="n"/>
@@ -992,7 +992,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Clinical Ops</t>
+          <t>Chemotherapy NS-2</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -1002,14 +1002,14 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Clinical Ops</t>
+          <t>Chemotherapy NS-2</t>
         </is>
       </c>
       <c r="D12" s="4" t="n"/>
       <c r="E12" s="4" t="n"/>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>1575</t>
+          <t>1282</t>
         </is>
       </c>
       <c r="G12" s="4" t="n"/>
@@ -1023,7 +1023,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Consultant Room 1- IVF</t>
+          <t>Chemotherapy- Doctor Room</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -1033,14 +1033,14 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Consultant Room 1- IVF</t>
+          <t>Chemotherapy- Doctor Room</t>
         </is>
       </c>
       <c r="D13" s="4" t="n"/>
       <c r="E13" s="4" t="n"/>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>1273</t>
+          <t>1270</t>
         </is>
       </c>
       <c r="G13" s="4" t="n"/>
@@ -1054,7 +1054,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Consultant Room 2- IVF</t>
+          <t>Clinical Ops</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -1064,14 +1064,14 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Consultant Room 2- IVF</t>
+          <t>Clinical Ops</t>
         </is>
       </c>
       <c r="D14" s="4" t="n"/>
       <c r="E14" s="4" t="n"/>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>1272</t>
+          <t>1575</t>
         </is>
       </c>
       <c r="G14" s="4" t="n"/>
@@ -1085,7 +1085,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Contact Centre</t>
+          <t>Consultant Room 1- IVF</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1095,14 +1095,14 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Contact Centre</t>
+          <t>Consultant Room 1- IVF</t>
         </is>
       </c>
       <c r="D15" s="4" t="n"/>
       <c r="E15" s="4" t="n"/>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>1670</t>
+          <t>1273</t>
         </is>
       </c>
       <c r="G15" s="4" t="n"/>
@@ -1116,7 +1116,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Contact Centre</t>
+          <t>Consultant Room 2- IVF</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1126,14 +1126,14 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Contact Centre</t>
+          <t>Consultant Room 2- IVF</t>
         </is>
       </c>
       <c r="D16" s="4" t="n"/>
       <c r="E16" s="4" t="n"/>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>1671</t>
+          <t>1272</t>
         </is>
       </c>
       <c r="G16" s="4" t="n"/>
@@ -1164,7 +1164,7 @@
       <c r="E17" s="4" t="n"/>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>1672</t>
+          <t>1670</t>
         </is>
       </c>
       <c r="G17" s="4" t="n"/>
@@ -1178,7 +1178,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Counselling Room- IVF</t>
+          <t>Contact Centre</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1188,14 +1188,14 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Counselling Room- IVF</t>
+          <t>Contact Centre</t>
         </is>
       </c>
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="4" t="n"/>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>1274</t>
+          <t>1671</t>
         </is>
       </c>
       <c r="G18" s="4" t="n"/>
@@ -1209,7 +1209,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Molly Thomas</t>
+          <t>Contact Centre</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1219,14 +1219,14 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>DNS</t>
+          <t>Contact Centre</t>
         </is>
       </c>
       <c r="D19" s="4" t="n"/>
       <c r="E19" s="4" t="n"/>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>1581</t>
+          <t>1672</t>
         </is>
       </c>
       <c r="G19" s="4" t="n"/>
@@ -1240,7 +1240,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Dailysis-Office</t>
+          <t>Counselling Room- IVF</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -1250,14 +1250,14 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Dailysis-Office</t>
+          <t>Counselling Room- IVF</t>
         </is>
       </c>
       <c r="D20" s="4" t="n"/>
       <c r="E20" s="4" t="n"/>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>1221</t>
+          <t>1274</t>
         </is>
       </c>
       <c r="G20" s="4" t="n"/>
@@ -1271,7 +1271,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Daycare - Main Reception</t>
+          <t>Molly Thomas</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -1281,14 +1281,14 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Daycare - Main Reception</t>
+          <t>DNS</t>
         </is>
       </c>
       <c r="D21" s="4" t="n"/>
       <c r="E21" s="4" t="n"/>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>1581</t>
         </is>
       </c>
       <c r="G21" s="4" t="n"/>
@@ -1302,7 +1302,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Daycare NS-1</t>
+          <t>Dailysis-Office</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -1312,14 +1312,14 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Daycare NS-1</t>
+          <t>Dailysis-Office</t>
         </is>
       </c>
       <c r="D22" s="4" t="n"/>
       <c r="E22" s="4" t="n"/>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>1284</t>
+          <t>1221</t>
         </is>
       </c>
       <c r="G22" s="4" t="n"/>
@@ -1333,7 +1333,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Daycare NS-1</t>
+          <t>Daycare - Main Reception</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -1343,14 +1343,14 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Daycare NS-1</t>
+          <t>Daycare - Main Reception</t>
         </is>
       </c>
       <c r="D23" s="4" t="n"/>
       <c r="E23" s="4" t="n"/>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>1285</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="G23" s="4" t="n"/>
@@ -1364,7 +1364,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Donor Counselling -Blood Bank</t>
+          <t>Daycare NS-1</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -1374,14 +1374,14 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Donor Counselling -Blood Bank</t>
+          <t>Daycare NS-1</t>
         </is>
       </c>
       <c r="D24" s="4" t="n"/>
       <c r="E24" s="4" t="n"/>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>1275</t>
+          <t>1284</t>
         </is>
       </c>
       <c r="G24" s="4" t="n"/>
@@ -1395,7 +1395,7 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Dr Devendra Kumar Agarwal room 143</t>
+          <t>Daycare NS-1</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -1405,14 +1405,14 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Dr Devendra Kumar Agarwal room 143</t>
+          <t>Daycare NS-1</t>
         </is>
       </c>
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>1143</t>
+          <t>1285</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -1426,7 +1426,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Dr Dharmesh L. Khatri room 125</t>
+          <t>Donor Counselling - Blood Bank</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -1436,14 +1436,14 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Dr Dharmesh L. Khatri room 125</t>
+          <t>Donor Counselling - Blood Bank</t>
         </is>
       </c>
       <c r="D26" s="4" t="n"/>
       <c r="E26" s="4" t="n"/>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>1125</t>
+          <t>1275</t>
         </is>
       </c>
       <c r="G26" s="4" t="n"/>
@@ -1457,7 +1457,7 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Dr Dibya Jyoti Mahakul room 121</t>
+          <t>Dr Devendra Kumar Agarwal room 143</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -1467,14 +1467,14 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Dr Dibya Jyoti Mahakul room 121</t>
+          <t>Dr Devendra Kumar Agarwal room 143</t>
         </is>
       </c>
       <c r="D27" s="4" t="n"/>
       <c r="E27" s="4" t="n"/>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>1121</t>
+          <t>1143</t>
         </is>
       </c>
       <c r="G27" s="4" t="n"/>
@@ -1488,7 +1488,7 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Dr Girraj Kishor Agarwal room 166</t>
+          <t>Dr Dharmesh L. Khatri room 125</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -1498,14 +1498,14 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Dr Girraj Kishor Agarwal room 166</t>
+          <t>Dr Dharmesh L. Khatri room 125</t>
         </is>
       </c>
       <c r="D28" s="4" t="n"/>
       <c r="E28" s="4" t="n"/>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>1166</t>
+          <t>1125</t>
         </is>
       </c>
       <c r="G28" s="4" t="n"/>
@@ -1519,7 +1519,7 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Dr Gurmeet Singh room 106</t>
+          <t>Dr Dibya Jyoti Mahakul room 121</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -1529,14 +1529,14 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Dr Gurmeet Singh room 106</t>
+          <t>Dr Dibya Jyoti Mahakul room 121</t>
         </is>
       </c>
       <c r="D29" s="4" t="n"/>
       <c r="E29" s="4" t="n"/>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>1106</t>
+          <t>1121</t>
         </is>
       </c>
       <c r="G29" s="4" t="n"/>
@@ -1550,7 +1550,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Dr Hanish Gupta room 108</t>
+          <t>Dr Girraj Kishor Agarwal room 166</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -1560,14 +1560,14 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Dr Hanish Gupta room 108</t>
+          <t>Dr Girraj Kishor Agarwal room 166</t>
         </is>
       </c>
       <c r="D30" s="4" t="n"/>
       <c r="E30" s="4" t="n"/>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>1108</t>
+          <t>1166</t>
         </is>
       </c>
       <c r="G30" s="4" t="n"/>
@@ -1581,7 +1581,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Dr Komal Sukhija room 111</t>
+          <t>Dr Gurmeet Singh room 106</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -1591,14 +1591,14 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Dr Komal Sukhija room 111</t>
+          <t>Dr Gurmeet Singh room 106</t>
         </is>
       </c>
       <c r="D31" s="4" t="n"/>
       <c r="E31" s="4" t="n"/>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>1111</t>
+          <t>1106</t>
         </is>
       </c>
       <c r="G31" s="4" t="n"/>
@@ -1612,7 +1612,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Dr Mandeep</t>
+          <t>Dr Hanish Gupta room 108</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -1622,14 +1622,14 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Dr Mandeep</t>
+          <t>Dr Hanish Gupta room 108</t>
         </is>
       </c>
       <c r="D32" s="4" t="n"/>
       <c r="E32" s="4" t="n"/>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>1075</t>
+          <t>1108</t>
         </is>
       </c>
       <c r="G32" s="4" t="n"/>
@@ -1643,7 +1643,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Dr Manmeet Kaur room 112</t>
+          <t>Dr Komal Sukhija room 111</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -1653,14 +1653,14 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Dr Manmeet Kaur room 112</t>
+          <t>Dr Komal Sukhija room 111</t>
         </is>
       </c>
       <c r="D33" s="4" t="n"/>
       <c r="E33" s="4" t="n"/>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>1112</t>
+          <t>1111</t>
         </is>
       </c>
       <c r="G33" s="4" t="n"/>
@@ -1674,7 +1674,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Dr Mohit Mann room 115</t>
+          <t>Dr Mandeep</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -1684,14 +1684,14 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Dr Mohit Mann room 115</t>
+          <t>Dr Mandeep</t>
         </is>
       </c>
       <c r="D34" s="4" t="n"/>
       <c r="E34" s="4" t="n"/>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>1115</t>
+          <t>1075</t>
         </is>
       </c>
       <c r="G34" s="4" t="n"/>
@@ -1705,7 +1705,7 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Dr Sandeep Kumar room 116</t>
+          <t>Dr Manmeet Kaur room 112</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -1715,14 +1715,14 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Dr Sandeep Kumar room 116</t>
+          <t>Dr Manmeet Kaur room 112</t>
         </is>
       </c>
       <c r="D35" s="4" t="n"/>
       <c r="E35" s="4" t="n"/>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>1116</t>
+          <t>1112</t>
         </is>
       </c>
       <c r="G35" s="4" t="n"/>
@@ -1736,7 +1736,7 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Dr Sanjeet Kumar Rai room 119</t>
+          <t>Dr Mohit Mann room 115</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -1746,14 +1746,14 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Dr Sanjeet Kumar Rai room 119</t>
+          <t>Dr Mohit Mann room 115</t>
         </is>
       </c>
       <c r="D36" s="4" t="n"/>
       <c r="E36" s="4" t="n"/>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>1119</t>
+          <t>1115</t>
         </is>
       </c>
       <c r="G36" s="4" t="n"/>
@@ -1767,7 +1767,7 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Dr Saurabh Mishra room 149</t>
+          <t>Dr Sandeep Kumar room 116</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -1777,14 +1777,14 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Dr Saurabh Mishra room 149</t>
+          <t>Dr Sandeep Kumar room 116</t>
         </is>
       </c>
       <c r="D37" s="4" t="n"/>
       <c r="E37" s="4" t="n"/>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>1149</t>
+          <t>1116</t>
         </is>
       </c>
       <c r="G37" s="4" t="n"/>
@@ -1798,7 +1798,7 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Dr Sonali Verma room105</t>
+          <t>Dr Sanjeet Kumar Rai room 119</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -1808,14 +1808,14 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Dr Sonali Verma room105</t>
+          <t>Dr Sanjeet Kumar Rai room 119</t>
         </is>
       </c>
       <c r="D38" s="4" t="n"/>
       <c r="E38" s="4" t="n"/>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>1105</t>
+          <t>1119</t>
         </is>
       </c>
       <c r="G38" s="4" t="n"/>
@@ -1829,7 +1829,7 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Dr Sumit room 127</t>
+          <t>Dr Saurabh Mishra room 149</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -1839,14 +1839,14 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Dr Sumit room 127</t>
+          <t>Dr Saurabh Mishra room 149</t>
         </is>
       </c>
       <c r="D39" s="4" t="n"/>
       <c r="E39" s="4" t="n"/>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>1127</t>
+          <t>1149</t>
         </is>
       </c>
       <c r="G39" s="4" t="n"/>
@@ -1860,7 +1860,7 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>Dr Sushil Kumar Mishra room 148</t>
+          <t>Dr Sonali Verma room105</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -1870,14 +1870,14 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Dr Sushil Kumar Mishra room 148</t>
+          <t>Dr Sonali Verma room105</t>
         </is>
       </c>
       <c r="D40" s="4" t="n"/>
       <c r="E40" s="4" t="n"/>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>1148</t>
+          <t>1105</t>
         </is>
       </c>
       <c r="G40" s="4" t="n"/>
@@ -1891,7 +1891,7 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>Dr Tushar Sharma room 120</t>
+          <t>Dr Sumit room 127</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
@@ -1901,14 +1901,14 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Dr Tushar Sharma room 120</t>
+          <t>Dr Sumit room 127</t>
         </is>
       </c>
       <c r="D41" s="4" t="n"/>
       <c r="E41" s="4" t="n"/>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>1120</t>
+          <t>1127</t>
         </is>
       </c>
       <c r="G41" s="4" t="n"/>
@@ -1922,7 +1922,7 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Dr Vandana Gulati Dhingra room 109</t>
+          <t>Dr Sushil Kumar Mishra room 148</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -1932,14 +1932,14 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Dr Vandana Gulati Dhingra room 109</t>
+          <t>Dr Sushil Kumar Mishra room 148</t>
         </is>
       </c>
       <c r="D42" s="4" t="n"/>
       <c r="E42" s="4" t="n"/>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>1109</t>
+          <t>1148</t>
         </is>
       </c>
       <c r="G42" s="4" t="n"/>
@@ -1953,7 +1953,7 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Dr. Naimaa K. Chaudhary room 164</t>
+          <t>Dr Tushar Sharma room 120</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -1963,14 +1963,14 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Dr. Naimaa K. Chaudhary room 164</t>
+          <t>Dr Tushar Sharma room 120</t>
         </is>
       </c>
       <c r="D43" s="4" t="n"/>
       <c r="E43" s="4" t="n"/>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>1164</t>
+          <t>1120</t>
         </is>
       </c>
       <c r="G43" s="4" t="n"/>
@@ -1984,7 +1984,7 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Dr. Nitin</t>
+          <t>Dr Vandana Gulati Dhingra room 109</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -1994,14 +1994,14 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Dr. Nitin</t>
+          <t>Dr Vandana Gulati Dhingra room 109</t>
         </is>
       </c>
       <c r="D44" s="4" t="n"/>
       <c r="E44" s="4" t="n"/>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>1576</t>
+          <t>1109</t>
         </is>
       </c>
       <c r="G44" s="4" t="n"/>
@@ -2015,7 +2015,7 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>Dr.(Prof.) Indu Chawla Chugh room 160</t>
+          <t>Dr. Naimaa K. Chaudhary room 164</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -2025,14 +2025,14 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Dr.(Prof.) Indu Chawla Chugh room 160</t>
+          <t>Dr. Naimaa K. Chaudhary room 164</t>
         </is>
       </c>
       <c r="D45" s="4" t="n"/>
       <c r="E45" s="4" t="n"/>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>1160</t>
+          <t>1164</t>
         </is>
       </c>
       <c r="G45" s="4" t="n"/>
@@ -2046,7 +2046,7 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>ER / Nursing Station</t>
+          <t>Dr. Nitin</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -2056,14 +2056,14 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>ER / Nursing Station</t>
+          <t>Dr. Nitin</t>
         </is>
       </c>
       <c r="D46" s="4" t="n"/>
       <c r="E46" s="4" t="n"/>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>1086</t>
+          <t>1576</t>
         </is>
       </c>
       <c r="G46" s="4" t="n"/>
@@ -2077,7 +2077,7 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>ER / Nursing Station</t>
+          <t>Dr.(Prof.) Indu Chawla Chugh room 160</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -2087,14 +2087,14 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>ER / Nursing Station</t>
+          <t>Dr.(Prof.) Indu Chawla Chugh room 160</t>
         </is>
       </c>
       <c r="D47" s="4" t="n"/>
       <c r="E47" s="4" t="n"/>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>1087</t>
+          <t>1160</t>
         </is>
       </c>
       <c r="G47" s="4" t="n"/>
@@ -2108,7 +2108,7 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>ER / Reception</t>
+          <t>ER / Nursing Station</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -2118,14 +2118,14 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>ER / Reception</t>
+          <t>ER / Nursing Station</t>
         </is>
       </c>
       <c r="D48" s="4" t="n"/>
       <c r="E48" s="4" t="n"/>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>1080</t>
+          <t>1086</t>
         </is>
       </c>
       <c r="G48" s="4" t="n"/>
@@ -2139,7 +2139,7 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>ER / Reception</t>
+          <t>ER / Nursing Station</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -2149,14 +2149,14 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>ER / Reception</t>
+          <t>ER / Nursing Station</t>
         </is>
       </c>
       <c r="D49" s="4" t="n"/>
       <c r="E49" s="4" t="n"/>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>1081</t>
+          <t>1087</t>
         </is>
       </c>
       <c r="G49" s="4" t="n"/>
@@ -2170,7 +2170,7 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>EWS Counter</t>
+          <t>ER / Reception</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -2180,14 +2180,14 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>EWS Counter</t>
+          <t>ER / Reception</t>
         </is>
       </c>
       <c r="D50" s="4" t="n"/>
       <c r="E50" s="4" t="n"/>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>1022</t>
+          <t>1080</t>
         </is>
       </c>
       <c r="G50" s="4" t="n"/>
@@ -2201,7 +2201,7 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>Saumen Malik</t>
+          <t>ER / Reception</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
@@ -2211,14 +2211,14 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>ER / Reception</t>
         </is>
       </c>
       <c r="D51" s="4" t="n"/>
       <c r="E51" s="4" t="n"/>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>1565</t>
+          <t>1081</t>
         </is>
       </c>
       <c r="G51" s="4" t="n"/>
@@ -2232,7 +2232,7 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>Shubhneet</t>
+          <t>EWS Counter</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -2242,14 +2242,14 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>EWS Counter</t>
         </is>
       </c>
       <c r="D52" s="4" t="n"/>
       <c r="E52" s="4" t="n"/>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>1564</t>
+          <t>1022</t>
         </is>
       </c>
       <c r="G52" s="4" t="n"/>
@@ -2263,7 +2263,7 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>Sohan</t>
+          <t>Saumen Malik</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -2280,7 +2280,7 @@
       <c r="E53" s="4" t="n"/>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>1061</t>
+          <t>1565</t>
         </is>
       </c>
       <c r="G53" s="4" t="n"/>
@@ -2294,7 +2294,7 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>Virender Rawat</t>
+          <t>Shubhneet</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -2311,7 +2311,7 @@
       <c r="E54" s="4" t="n"/>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>1060</t>
+          <t>1564</t>
         </is>
       </c>
       <c r="G54" s="4" t="n"/>
@@ -2325,7 +2325,7 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>Fire Control Room</t>
+          <t>Sohan</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -2335,14 +2335,14 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Fire Control Room</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D55" s="4" t="n"/>
       <c r="E55" s="4" t="n"/>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>1099</t>
+          <t>1061</t>
         </is>
       </c>
       <c r="G55" s="4" t="n"/>
@@ -2356,7 +2356,7 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>Aditya Rai</t>
+          <t>Virender Rawat</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -2366,14 +2366,14 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D56" s="4" t="n"/>
       <c r="E56" s="4" t="n"/>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>1528</t>
+          <t>1060</t>
         </is>
       </c>
       <c r="G56" s="4" t="n"/>
@@ -2387,7 +2387,7 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>Ashmita Sethi</t>
+          <t>Fire Control Room</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -2397,14 +2397,14 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Fire Control Room</t>
         </is>
       </c>
       <c r="D57" s="4" t="n"/>
       <c r="E57" s="4" t="n"/>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>1099</t>
         </is>
       </c>
       <c r="G57" s="4" t="n"/>
@@ -2418,7 +2418,7 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>Dr Saloni Jindal</t>
+          <t>Aditya Rai</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -2435,7 +2435,7 @@
       <c r="E58" s="4" t="n"/>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>1527</t>
+          <t>1528</t>
         </is>
       </c>
       <c r="G58" s="4" t="n"/>
@@ -2449,7 +2449,7 @@
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>Sabyasachi Roy</t>
+          <t>Ashmita Sethi</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -2466,7 +2466,7 @@
       <c r="E59" s="4" t="n"/>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>1525</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="G59" s="4" t="n"/>
@@ -2480,7 +2480,7 @@
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>Shivani</t>
+          <t>Dr Saloni Jindal</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -2497,7 +2497,7 @@
       <c r="E60" s="4" t="n"/>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>1526</t>
+          <t>1527</t>
         </is>
       </c>
       <c r="G60" s="4" t="n"/>
@@ -2511,7 +2511,7 @@
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>Head -IT</t>
+          <t>Sabyasachi Roy</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -2521,14 +2521,14 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Head -IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D61" s="4" t="n"/>
       <c r="E61" s="4" t="n"/>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>1550</t>
+          <t>1525</t>
         </is>
       </c>
       <c r="G61" s="4" t="n"/>
@@ -2542,7 +2542,7 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>Healthcheckup Reception</t>
+          <t>Shivani</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -2552,14 +2552,14 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Healthcheckup Reception</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D62" s="4" t="n"/>
       <c r="E62" s="4" t="n"/>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>1070</t>
+          <t>1526</t>
         </is>
       </c>
       <c r="G62" s="4" t="n"/>
@@ -2573,7 +2573,7 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>Histopathlogy Consultant Room</t>
+          <t>Head -IT</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
@@ -2583,14 +2583,14 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Histopathlogy Consultant Room</t>
+          <t>Head -IT</t>
         </is>
       </c>
       <c r="D63" s="4" t="n"/>
       <c r="E63" s="4" t="n"/>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>1253</t>
+          <t>1550</t>
         </is>
       </c>
       <c r="G63" s="4" t="n"/>
@@ -2604,7 +2604,7 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>IP Admission</t>
+          <t>Healthcheckup Reception</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -2614,14 +2614,14 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>IP Admission</t>
+          <t>Healthcheckup Reception</t>
         </is>
       </c>
       <c r="D64" s="4" t="n"/>
       <c r="E64" s="4" t="n"/>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>1065</t>
+          <t>1070</t>
         </is>
       </c>
       <c r="G64" s="4" t="n"/>
@@ -2635,7 +2635,7 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>IP Admission</t>
+          <t>Histopathlogy Consultant Room</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
@@ -2645,14 +2645,14 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>IP Admission</t>
+          <t>Histopathlogy Consultant Room</t>
         </is>
       </c>
       <c r="D65" s="4" t="n"/>
       <c r="E65" s="4" t="n"/>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>1066</t>
+          <t>1253</t>
         </is>
       </c>
       <c r="G65" s="4" t="n"/>
@@ -2683,7 +2683,7 @@
       <c r="E66" s="4" t="n"/>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>1067</t>
+          <t>1065</t>
         </is>
       </c>
       <c r="G66" s="4" t="n"/>
@@ -2714,7 +2714,7 @@
       <c r="E67" s="4" t="n"/>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>1068</t>
+          <t>1066</t>
         </is>
       </c>
       <c r="G67" s="4" t="n"/>
@@ -2745,7 +2745,7 @@
       <c r="E68" s="4" t="n"/>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>1069</t>
+          <t>1067</t>
         </is>
       </c>
       <c r="G68" s="4" t="n"/>
@@ -2759,7 +2759,7 @@
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>IVF- Reception</t>
+          <t>IP Admission</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
@@ -2769,14 +2769,14 @@
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>IVF- Reception</t>
+          <t>IP Admission</t>
         </is>
       </c>
       <c r="D69" s="4" t="n"/>
       <c r="E69" s="4" t="n"/>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>1203</t>
+          <t>1068</t>
         </is>
       </c>
       <c r="G69" s="4" t="n"/>
@@ -2790,7 +2790,7 @@
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>Investigation Counter</t>
+          <t>IP Admission</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
@@ -2800,14 +2800,14 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Investigation Counter</t>
+          <t>IP Admission</t>
         </is>
       </c>
       <c r="D70" s="4" t="n"/>
       <c r="E70" s="4" t="n"/>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>1069</t>
         </is>
       </c>
       <c r="G70" s="4" t="n"/>
@@ -2821,7 +2821,7 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>Harjeet Singh Bhalla</t>
+          <t>IT Staff</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
@@ -2831,14 +2831,14 @@
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Legal</t>
+          <t>IT Staff</t>
         </is>
       </c>
       <c r="D71" s="4" t="n"/>
       <c r="E71" s="4" t="n"/>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>1516</t>
+          <t>1553</t>
         </is>
       </c>
       <c r="G71" s="4" t="n"/>
@@ -2852,7 +2852,7 @@
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>Main Reception / H24 Help</t>
+          <t>IT Staff</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
@@ -2862,14 +2862,14 @@
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Main Reception / H24 Help</t>
+          <t>IT Staff</t>
         </is>
       </c>
       <c r="D72" s="4" t="n"/>
       <c r="E72" s="4" t="n"/>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>1500</t>
+          <t>1554</t>
         </is>
       </c>
       <c r="G72" s="4" t="n"/>
@@ -2883,24 +2883,24 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>CCS</t>
+          <t>IT Staff</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>CCS</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>Management Team</t>
+          <t>IT Staff</t>
         </is>
       </c>
       <c r="D73" s="4" t="n"/>
       <c r="E73" s="4" t="n"/>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>1570</t>
+          <t>1555</t>
         </is>
       </c>
       <c r="G73" s="4" t="n"/>
@@ -2914,24 +2914,24 @@
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>IT Staff</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>CEO</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>Management Team</t>
+          <t>IT Staff</t>
         </is>
       </c>
       <c r="D74" s="4" t="n"/>
       <c r="E74" s="4" t="n"/>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>1510</t>
+          <t>1556</t>
         </is>
       </c>
       <c r="G74" s="4" t="n"/>
@@ -2945,24 +2945,24 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>CFO</t>
+          <t>IT Staff</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>CFO</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>Management Team</t>
+          <t>IT Staff</t>
         </is>
       </c>
       <c r="D75" s="4" t="n"/>
       <c r="E75" s="4" t="n"/>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>1560</t>
+          <t>1557</t>
         </is>
       </c>
       <c r="G75" s="4" t="n"/>
@@ -2976,24 +2976,24 @@
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>CMO</t>
+          <t>IT Staff</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>CMO</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Management Team</t>
+          <t>IT Staff</t>
         </is>
       </c>
       <c r="D76" s="4" t="n"/>
       <c r="E76" s="4" t="n"/>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>1011</t>
+          <t>1558</t>
         </is>
       </c>
       <c r="G76" s="4" t="n"/>
@@ -3007,24 +3007,24 @@
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>CNO</t>
+          <t>IVF- Reception</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>CNO</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Management Team</t>
+          <t>IVF- Reception</t>
         </is>
       </c>
       <c r="D77" s="4" t="n"/>
       <c r="E77" s="4" t="n"/>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>1580</t>
+          <t>1203</t>
         </is>
       </c>
       <c r="G77" s="4" t="n"/>
@@ -3038,24 +3038,24 @@
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>COO</t>
+          <t>Investigation Counter</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>COO</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Management Team</t>
+          <t>Investigation Counter</t>
         </is>
       </c>
       <c r="D78" s="4" t="n"/>
       <c r="E78" s="4" t="n"/>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>1520</t>
+          <t>1100</t>
         </is>
       </c>
       <c r="G78" s="4" t="n"/>
@@ -3069,24 +3069,24 @@
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>Vishal Rao</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Management Team</t>
+          <t>Lead Contact Centre</t>
         </is>
       </c>
       <c r="D79" s="4" t="n"/>
       <c r="E79" s="4" t="n"/>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>1010</t>
+          <t>5678</t>
         </is>
       </c>
       <c r="G79" s="4" t="n"/>
@@ -3100,7 +3100,7 @@
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>Manager Operations</t>
+          <t>Harjeet Singh Bhalla</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
@@ -3110,14 +3110,14 @@
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Manager Operations</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="D80" s="4" t="n"/>
       <c r="E80" s="4" t="n"/>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>1533</t>
+          <t>1516</t>
         </is>
       </c>
       <c r="G80" s="4" t="n"/>
@@ -3131,7 +3131,7 @@
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>Manisha -HR Helpdesk</t>
+          <t>Main Reception / H24 Help</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
@@ -3141,14 +3141,14 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Manisha -HR Helpdesk</t>
+          <t>Main Reception / H24 Help</t>
         </is>
       </c>
       <c r="D81" s="4" t="n"/>
       <c r="E81" s="4" t="n"/>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>1577</t>
+          <t>1500</t>
         </is>
       </c>
       <c r="G81" s="4" t="n"/>
@@ -3162,24 +3162,24 @@
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>CCS</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>CCS</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Management Team</t>
         </is>
       </c>
       <c r="D82" s="4" t="n"/>
       <c r="E82" s="4" t="n"/>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>1531</t>
+          <t>1570</t>
         </is>
       </c>
       <c r="G82" s="4" t="n"/>
@@ -3193,24 +3193,24 @@
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Management Team</t>
         </is>
       </c>
       <c r="D83" s="4" t="n"/>
       <c r="E83" s="4" t="n"/>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>1532</t>
+          <t>1510</t>
         </is>
       </c>
       <c r="G83" s="4" t="n"/>
@@ -3224,24 +3224,24 @@
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>Rahul Arora</t>
+          <t>CFO</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>CFO</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Management Team</t>
         </is>
       </c>
       <c r="D84" s="4" t="n"/>
       <c r="E84" s="4" t="n"/>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>1530</t>
+          <t>1560</t>
         </is>
       </c>
       <c r="G84" s="4" t="n"/>
@@ -3255,24 +3255,24 @@
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>Microbiology Consultant Room</t>
+          <t>CMO</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>CMO</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Microbiology Consultant Room</t>
+          <t>Management Team</t>
         </is>
       </c>
       <c r="D85" s="4" t="n"/>
       <c r="E85" s="4" t="n"/>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>1254</t>
+          <t>1011</t>
         </is>
       </c>
       <c r="G85" s="4" t="n"/>
@@ -3286,24 +3286,24 @@
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>Nursing Station -3</t>
+          <t>CNO</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>CNO</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Nursing Station -3</t>
+          <t>Management Team</t>
         </is>
       </c>
       <c r="D86" s="4" t="n"/>
       <c r="E86" s="4" t="n"/>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>1183</t>
+          <t>1580</t>
         </is>
       </c>
       <c r="G86" s="4" t="n"/>
@@ -3317,24 +3317,24 @@
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>OPD Pharmacy</t>
+          <t>COO</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>COO</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>OPD Pharmacy</t>
+          <t>Management Team</t>
         </is>
       </c>
       <c r="D87" s="4" t="n"/>
       <c r="E87" s="4" t="n"/>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>1161</t>
+          <t>1520</t>
         </is>
       </c>
       <c r="G87" s="4" t="n"/>
@@ -3348,24 +3348,24 @@
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>OPD Pharmacy</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>OPD Pharmacy</t>
+          <t>Management Team</t>
         </is>
       </c>
       <c r="D88" s="4" t="n"/>
       <c r="E88" s="4" t="n"/>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>1162</t>
+          <t>1010</t>
         </is>
       </c>
       <c r="G88" s="4" t="n"/>
@@ -3379,7 +3379,7 @@
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 104</t>
+          <t>Manager Operations</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
@@ -3389,14 +3389,14 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 104</t>
+          <t>Manager Operations</t>
         </is>
       </c>
       <c r="D89" s="4" t="n"/>
       <c r="E89" s="4" t="n"/>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>1104</t>
+          <t>1533</t>
         </is>
       </c>
       <c r="G89" s="4" t="n"/>
@@ -3410,7 +3410,7 @@
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 107</t>
+          <t>Manisha -HR Helpdesk</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
@@ -3420,14 +3420,14 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 107</t>
+          <t>Manisha -HR Helpdesk</t>
         </is>
       </c>
       <c r="D90" s="4" t="n"/>
       <c r="E90" s="4" t="n"/>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>1107</t>
+          <t>1577</t>
         </is>
       </c>
       <c r="G90" s="4" t="n"/>
@@ -3441,7 +3441,7 @@
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 113</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
@@ -3451,14 +3451,14 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 113</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D91" s="4" t="n"/>
       <c r="E91" s="4" t="n"/>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>1113</t>
+          <t>1531</t>
         </is>
       </c>
       <c r="G91" s="4" t="n"/>
@@ -3472,7 +3472,7 @@
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 114</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
@@ -3482,14 +3482,14 @@
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 114</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D92" s="4" t="n"/>
       <c r="E92" s="4" t="n"/>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>1114</t>
+          <t>1532</t>
         </is>
       </c>
       <c r="G92" s="4" t="n"/>
@@ -3503,7 +3503,7 @@
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 122</t>
+          <t>Rahul Arora</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
@@ -3513,14 +3513,14 @@
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 122</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D93" s="4" t="n"/>
       <c r="E93" s="4" t="n"/>
       <c r="F93" s="4" t="inlineStr">
         <is>
-          <t>1122</t>
+          <t>1530</t>
         </is>
       </c>
       <c r="G93" s="4" t="n"/>
@@ -3534,7 +3534,7 @@
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 123</t>
+          <t>Microbiology Consultant Room</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
@@ -3544,14 +3544,14 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 123</t>
+          <t>Microbiology Consultant Room</t>
         </is>
       </c>
       <c r="D94" s="4" t="n"/>
       <c r="E94" s="4" t="n"/>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>1123</t>
+          <t>1254</t>
         </is>
       </c>
       <c r="G94" s="4" t="n"/>
@@ -3565,7 +3565,7 @@
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 128</t>
+          <t>Nursing Station -3</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
@@ -3575,14 +3575,14 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 128</t>
+          <t>Nursing Station -3</t>
         </is>
       </c>
       <c r="D95" s="4" t="n"/>
       <c r="E95" s="4" t="n"/>
       <c r="F95" s="4" t="inlineStr">
         <is>
-          <t>1128</t>
+          <t>1183</t>
         </is>
       </c>
       <c r="G95" s="4" t="n"/>
@@ -3596,7 +3596,7 @@
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 129</t>
+          <t>OPD Pharmacy</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
@@ -3606,14 +3606,14 @@
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 129</t>
+          <t>OPD Pharmacy</t>
         </is>
       </c>
       <c r="D96" s="4" t="n"/>
       <c r="E96" s="4" t="n"/>
       <c r="F96" s="4" t="inlineStr">
         <is>
-          <t>1129</t>
+          <t>1161</t>
         </is>
       </c>
       <c r="G96" s="4" t="n"/>
@@ -3627,7 +3627,7 @@
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 130</t>
+          <t>OPD Pharmacy</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
@@ -3637,14 +3637,14 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 130</t>
+          <t>OPD Pharmacy</t>
         </is>
       </c>
       <c r="D97" s="4" t="n"/>
       <c r="E97" s="4" t="n"/>
       <c r="F97" s="4" t="inlineStr">
         <is>
-          <t>1130</t>
+          <t>1162</t>
         </is>
       </c>
       <c r="G97" s="4" t="n"/>
@@ -3658,7 +3658,7 @@
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 141</t>
+          <t>OPD room 122</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
@@ -3668,14 +3668,14 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 141</t>
+          <t>OPD room 122</t>
         </is>
       </c>
       <c r="D98" s="4" t="n"/>
       <c r="E98" s="4" t="n"/>
       <c r="F98" s="4" t="inlineStr">
         <is>
-          <t>1141</t>
+          <t>1122</t>
         </is>
       </c>
       <c r="G98" s="4" t="n"/>
@@ -3689,7 +3689,7 @@
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 144</t>
+          <t>OPD room 128</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
@@ -3699,14 +3699,14 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 144</t>
+          <t>OPD room 128</t>
         </is>
       </c>
       <c r="D99" s="4" t="n"/>
       <c r="E99" s="4" t="n"/>
       <c r="F99" s="4" t="inlineStr">
         <is>
-          <t>1144</t>
+          <t>1128</t>
         </is>
       </c>
       <c r="G99" s="4" t="n"/>
@@ -3720,7 +3720,7 @@
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 145</t>
+          <t>OPD room 129</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
@@ -3730,14 +3730,14 @@
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 145</t>
+          <t>OPD room 129</t>
         </is>
       </c>
       <c r="D100" s="4" t="n"/>
       <c r="E100" s="4" t="n"/>
       <c r="F100" s="4" t="inlineStr">
         <is>
-          <t>1145</t>
+          <t>1129</t>
         </is>
       </c>
       <c r="G100" s="4" t="n"/>
@@ -3751,7 +3751,7 @@
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 150</t>
+          <t>OPD room 130</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
@@ -3761,14 +3761,14 @@
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 150</t>
+          <t>OPD room 130</t>
         </is>
       </c>
       <c r="D101" s="4" t="n"/>
       <c r="E101" s="4" t="n"/>
       <c r="F101" s="4" t="inlineStr">
         <is>
-          <t>1150</t>
+          <t>1130</t>
         </is>
       </c>
       <c r="G101" s="4" t="n"/>
@@ -3782,7 +3782,7 @@
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 151</t>
+          <t>OPD room 141</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
@@ -3792,14 +3792,14 @@
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 151</t>
+          <t>OPD room 141</t>
         </is>
       </c>
       <c r="D102" s="4" t="n"/>
       <c r="E102" s="4" t="n"/>
       <c r="F102" s="4" t="inlineStr">
         <is>
-          <t>1151</t>
+          <t>1141</t>
         </is>
       </c>
       <c r="G102" s="4" t="n"/>
@@ -3813,7 +3813,7 @@
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 152</t>
+          <t>OPD room 144</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
@@ -3823,14 +3823,14 @@
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 152</t>
+          <t>OPD room 144</t>
         </is>
       </c>
       <c r="D103" s="4" t="n"/>
       <c r="E103" s="4" t="n"/>
       <c r="F103" s="4" t="inlineStr">
         <is>
-          <t>1152</t>
+          <t>1144</t>
         </is>
       </c>
       <c r="G103" s="4" t="n"/>
@@ -3844,7 +3844,7 @@
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 153</t>
+          <t>OPD room 145</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
@@ -3854,14 +3854,14 @@
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 153</t>
+          <t>OPD room 145</t>
         </is>
       </c>
       <c r="D104" s="4" t="n"/>
       <c r="E104" s="4" t="n"/>
       <c r="F104" s="4" t="inlineStr">
         <is>
-          <t>1153</t>
+          <t>1145</t>
         </is>
       </c>
       <c r="G104" s="4" t="n"/>
@@ -3875,7 +3875,7 @@
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 155</t>
+          <t>OPD room 150</t>
         </is>
       </c>
       <c r="B105" s="4" t="inlineStr">
@@ -3885,14 +3885,14 @@
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>OPD room No 155</t>
+          <t>OPD room 150</t>
         </is>
       </c>
       <c r="D105" s="4" t="n"/>
       <c r="E105" s="4" t="n"/>
       <c r="F105" s="4" t="inlineStr">
         <is>
-          <t>1155</t>
+          <t>1150</t>
         </is>
       </c>
       <c r="G105" s="4" t="n"/>
@@ -3906,7 +3906,7 @@
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>Anuradha</t>
+          <t>OPD room 151</t>
         </is>
       </c>
       <c r="B106" s="4" t="inlineStr">
@@ -3916,14 +3916,14 @@
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>OPD room 151</t>
         </is>
       </c>
       <c r="D106" s="4" t="n"/>
       <c r="E106" s="4" t="n"/>
       <c r="F106" s="4" t="inlineStr">
         <is>
-          <t>1522</t>
+          <t>1151</t>
         </is>
       </c>
       <c r="G106" s="4" t="n"/>
@@ -3937,7 +3937,7 @@
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>Ausaf Alam</t>
+          <t>OPD room 152</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
@@ -3947,14 +3947,14 @@
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>OPD room 152</t>
         </is>
       </c>
       <c r="D107" s="4" t="n"/>
       <c r="E107" s="4" t="n"/>
       <c r="F107" s="4" t="inlineStr">
         <is>
-          <t>1523</t>
+          <t>1152</t>
         </is>
       </c>
       <c r="G107" s="4" t="n"/>
@@ -3968,7 +3968,7 @@
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>Rahul Sharma</t>
+          <t>OPD room 153</t>
         </is>
       </c>
       <c r="B108" s="4" t="inlineStr">
@@ -3978,14 +3978,14 @@
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>OPD room 153</t>
         </is>
       </c>
       <c r="D108" s="4" t="n"/>
       <c r="E108" s="4" t="n"/>
       <c r="F108" s="4" t="inlineStr">
         <is>
-          <t>1524</t>
+          <t>1153</t>
         </is>
       </c>
       <c r="G108" s="4" t="n"/>
@@ -3999,7 +3999,7 @@
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>Vipin Dhawan</t>
+          <t>OPD room 155</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
@@ -4009,14 +4009,14 @@
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>OPD room 155</t>
         </is>
       </c>
       <c r="D109" s="4" t="n"/>
       <c r="E109" s="4" t="n"/>
       <c r="F109" s="4" t="inlineStr">
         <is>
-          <t>1521</t>
+          <t>1155</t>
         </is>
       </c>
       <c r="G109" s="4" t="n"/>
@@ -4030,7 +4030,7 @@
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>Ops team</t>
+          <t>OPD room104</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
@@ -4040,14 +4040,14 @@
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>Ops team</t>
+          <t>OPD room104</t>
         </is>
       </c>
       <c r="D110" s="4" t="n"/>
       <c r="E110" s="4" t="n"/>
       <c r="F110" s="4" t="inlineStr">
         <is>
-          <t>1534</t>
+          <t>1104</t>
         </is>
       </c>
       <c r="G110" s="4" t="n"/>
@@ -4061,7 +4061,7 @@
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>Salina</t>
+          <t>OPD room107</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
@@ -4071,14 +4071,14 @@
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>PHC</t>
+          <t>OPD room107</t>
         </is>
       </c>
       <c r="D111" s="4" t="n"/>
       <c r="E111" s="4" t="n"/>
       <c r="F111" s="4" t="inlineStr">
         <is>
-          <t>1074</t>
+          <t>1107</t>
         </is>
       </c>
       <c r="G111" s="4" t="n"/>
@@ -4092,7 +4092,7 @@
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>PICU Nursing Station</t>
+          <t>OPD room113</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
@@ -4102,14 +4102,14 @@
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>PICU Nursing Station</t>
+          <t>OPD room113</t>
         </is>
       </c>
       <c r="D112" s="4" t="n"/>
       <c r="E112" s="4" t="n"/>
       <c r="F112" s="4" t="inlineStr">
         <is>
-          <t>1380</t>
+          <t>1113</t>
         </is>
       </c>
       <c r="G112" s="4" t="n"/>
@@ -4123,7 +4123,7 @@
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>PRO</t>
+          <t>OPD room114</t>
         </is>
       </c>
       <c r="B113" s="4" t="inlineStr">
@@ -4133,14 +4133,14 @@
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>PRO</t>
+          <t>OPD room114</t>
         </is>
       </c>
       <c r="D113" s="4" t="n"/>
       <c r="E113" s="4" t="n"/>
       <c r="F113" s="4" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>1114</t>
         </is>
       </c>
       <c r="G113" s="4" t="n"/>
@@ -4154,7 +4154,7 @@
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>PRO</t>
+          <t>OPD room123</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
@@ -4164,14 +4164,14 @@
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>PRO</t>
+          <t>OPD room123</t>
         </is>
       </c>
       <c r="D114" s="4" t="n"/>
       <c r="E114" s="4" t="n"/>
       <c r="F114" s="4" t="inlineStr">
         <is>
-          <t>1103</t>
+          <t>1123</t>
         </is>
       </c>
       <c r="G114" s="4" t="n"/>
@@ -4185,7 +4185,7 @@
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t>Pathlogy Consultant Room</t>
+          <t>Anuradha</t>
         </is>
       </c>
       <c r="B115" s="4" t="inlineStr">
@@ -4195,14 +4195,14 @@
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>Pathlogy Consultant Room</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="D115" s="4" t="n"/>
       <c r="E115" s="4" t="n"/>
       <c r="F115" s="4" t="inlineStr">
         <is>
-          <t>1252</t>
+          <t>1522</t>
         </is>
       </c>
       <c r="G115" s="4" t="n"/>
@@ -4216,7 +4216,7 @@
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>Deepak Khurana</t>
+          <t>Ausaf Alam</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
@@ -4226,14 +4226,14 @@
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>Pharmacy</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="D116" s="4" t="n"/>
       <c r="E116" s="4" t="n"/>
       <c r="F116" s="4" t="inlineStr">
         <is>
-          <t>1566</t>
+          <t>1523</t>
         </is>
       </c>
       <c r="G116" s="4" t="n"/>
@@ -4247,7 +4247,7 @@
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>Nitesh Raghav</t>
+          <t>Rahul Sharma</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
@@ -4257,14 +4257,14 @@
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>Pharmacy</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="D117" s="4" t="n"/>
       <c r="E117" s="4" t="n"/>
       <c r="F117" s="4" t="inlineStr">
         <is>
-          <t>1567</t>
+          <t>1524</t>
         </is>
       </c>
       <c r="G117" s="4" t="n"/>
@@ -4278,7 +4278,7 @@
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>Divya Kataria</t>
+          <t>Vipin Dhawan</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
@@ -4288,14 +4288,14 @@
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>Physiotherapy</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="D118" s="4" t="n"/>
       <c r="E118" s="4" t="n"/>
       <c r="F118" s="4" t="inlineStr">
         <is>
-          <t>1568</t>
+          <t>1521</t>
         </is>
       </c>
       <c r="G118" s="4" t="n"/>
@@ -4309,7 +4309,7 @@
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>Physiotherapy</t>
+          <t>Ops team</t>
         </is>
       </c>
       <c r="B119" s="4" t="inlineStr">
@@ -4319,14 +4319,14 @@
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>Physiotherapy</t>
+          <t>Ops team</t>
         </is>
       </c>
       <c r="D119" s="4" t="n"/>
       <c r="E119" s="4" t="n"/>
       <c r="F119" s="4" t="inlineStr">
         <is>
-          <t>1230</t>
+          <t>1534</t>
         </is>
       </c>
       <c r="G119" s="4" t="n"/>
@@ -4340,7 +4340,7 @@
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>Physiotherapy</t>
+          <t>Salina</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
@@ -4350,14 +4350,14 @@
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>Physiotherapy</t>
+          <t>PHC</t>
         </is>
       </c>
       <c r="D120" s="4" t="n"/>
       <c r="E120" s="4" t="n"/>
       <c r="F120" s="4" t="inlineStr">
         <is>
-          <t>1231</t>
+          <t>1074</t>
         </is>
       </c>
       <c r="G120" s="4" t="n"/>
@@ -4371,7 +4371,7 @@
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>Physiotherapy</t>
+          <t>PICU Nursing Station</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
@@ -4381,14 +4381,14 @@
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>Physiotherapy</t>
+          <t>PICU Nursing Station</t>
         </is>
       </c>
       <c r="D121" s="4" t="n"/>
       <c r="E121" s="4" t="n"/>
       <c r="F121" s="4" t="inlineStr">
         <is>
-          <t>1233</t>
+          <t>1380</t>
         </is>
       </c>
       <c r="G121" s="4" t="n"/>
@@ -4402,7 +4402,7 @@
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>Physiotherapy - Main Reception</t>
+          <t>PRO</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr">
@@ -4412,14 +4412,14 @@
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>Physiotherapy - Main Reception</t>
+          <t>PRO</t>
         </is>
       </c>
       <c r="D122" s="4" t="n"/>
       <c r="E122" s="4" t="n"/>
       <c r="F122" s="4" t="inlineStr">
         <is>
-          <t>1201</t>
+          <t>1003</t>
         </is>
       </c>
       <c r="G122" s="4" t="n"/>
@@ -4433,7 +4433,7 @@
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>Himanshu Nath</t>
+          <t>PRO</t>
         </is>
       </c>
       <c r="B123" s="4" t="inlineStr">
@@ -4443,14 +4443,14 @@
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>PRO</t>
         </is>
       </c>
       <c r="D123" s="4" t="n"/>
       <c r="E123" s="4" t="n"/>
       <c r="F123" s="4" t="inlineStr">
         <is>
-          <t>1515</t>
+          <t>1103</t>
         </is>
       </c>
       <c r="G123" s="4" t="n"/>
@@ -4464,7 +4464,7 @@
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
         <is>
-          <t>Radiologist 1</t>
+          <t>Pathlogy Consultant Room</t>
         </is>
       </c>
       <c r="B124" s="4" t="inlineStr">
@@ -4474,14 +4474,14 @@
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>Radiologist 1</t>
+          <t>Pathlogy Consultant Room</t>
         </is>
       </c>
       <c r="D124" s="4" t="n"/>
       <c r="E124" s="4" t="n"/>
       <c r="F124" s="4" t="inlineStr">
         <is>
-          <t>1034</t>
+          <t>1252</t>
         </is>
       </c>
       <c r="G124" s="4" t="n"/>
@@ -4495,7 +4495,7 @@
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
         <is>
-          <t>Radiology reception</t>
+          <t>Deepak Khurana</t>
         </is>
       </c>
       <c r="B125" s="4" t="inlineStr">
@@ -4505,14 +4505,14 @@
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>Radiology reception</t>
+          <t>Pharmacy</t>
         </is>
       </c>
       <c r="D125" s="4" t="n"/>
       <c r="E125" s="4" t="n"/>
       <c r="F125" s="4" t="inlineStr">
         <is>
-          <t>1030</t>
+          <t>1566</t>
         </is>
       </c>
       <c r="G125" s="4" t="n"/>
@@ -4526,7 +4526,7 @@
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
         <is>
-          <t>Radiology reception</t>
+          <t>Nitesh Raghav</t>
         </is>
       </c>
       <c r="B126" s="4" t="inlineStr">
@@ -4536,14 +4536,14 @@
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>Radiology reception</t>
+          <t>Pharmacy</t>
         </is>
       </c>
       <c r="D126" s="4" t="n"/>
       <c r="E126" s="4" t="n"/>
       <c r="F126" s="4" t="inlineStr">
         <is>
-          <t>1031</t>
+          <t>1567</t>
         </is>
       </c>
       <c r="G126" s="4" t="n"/>
@@ -4557,7 +4557,7 @@
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
         <is>
-          <t>Registration Counter</t>
+          <t>Divya Kataria</t>
         </is>
       </c>
       <c r="B127" s="4" t="inlineStr">
@@ -4567,14 +4567,14 @@
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>Registration Counter</t>
+          <t>Physiotherapy</t>
         </is>
       </c>
       <c r="D127" s="4" t="n"/>
       <c r="E127" s="4" t="n"/>
       <c r="F127" s="4" t="inlineStr">
         <is>
-          <t>1165</t>
+          <t>1568</t>
         </is>
       </c>
       <c r="G127" s="4" t="n"/>
@@ -4588,7 +4588,7 @@
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
         <is>
-          <t>Registration Counter</t>
+          <t>Physiotherapy</t>
         </is>
       </c>
       <c r="B128" s="4" t="inlineStr">
@@ -4598,14 +4598,14 @@
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>Registration Counter</t>
+          <t>Physiotherapy</t>
         </is>
       </c>
       <c r="D128" s="4" t="n"/>
       <c r="E128" s="4" t="n"/>
       <c r="F128" s="4" t="inlineStr">
         <is>
-          <t>1167</t>
+          <t>1230</t>
         </is>
       </c>
       <c r="G128" s="4" t="n"/>
@@ -4619,7 +4619,7 @@
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
         <is>
-          <t>Registration Counter</t>
+          <t>Physiotherapy</t>
         </is>
       </c>
       <c r="B129" s="4" t="inlineStr">
@@ -4629,14 +4629,14 @@
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>Registration Counter</t>
+          <t>Physiotherapy</t>
         </is>
       </c>
       <c r="D129" s="4" t="n"/>
       <c r="E129" s="4" t="n"/>
       <c r="F129" s="4" t="inlineStr">
         <is>
-          <t>1168</t>
+          <t>1231</t>
         </is>
       </c>
       <c r="G129" s="4" t="n"/>
@@ -4650,7 +4650,7 @@
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>Registration Counter</t>
+          <t>Physiotherapy</t>
         </is>
       </c>
       <c r="B130" s="4" t="inlineStr">
@@ -4660,14 +4660,14 @@
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>Registration Counter</t>
+          <t>Physiotherapy</t>
         </is>
       </c>
       <c r="D130" s="4" t="n"/>
       <c r="E130" s="4" t="n"/>
       <c r="F130" s="4" t="inlineStr">
         <is>
-          <t>1169</t>
+          <t>1233</t>
         </is>
       </c>
       <c r="G130" s="4" t="n"/>
@@ -4681,7 +4681,7 @@
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>Adil</t>
+          <t>Physiotherapy - Main Reception</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
@@ -4691,14 +4691,14 @@
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>SCM</t>
+          <t>Physiotherapy - Main Reception</t>
         </is>
       </c>
       <c r="D131" s="4" t="n"/>
       <c r="E131" s="4" t="n"/>
       <c r="F131" s="4" t="inlineStr">
         <is>
-          <t>1539</t>
+          <t>1201</t>
         </is>
       </c>
       <c r="G131" s="4" t="n"/>
@@ -4712,7 +4712,7 @@
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t>Rajeev Kumar Malik</t>
+          <t>Himanshu Nath</t>
         </is>
       </c>
       <c r="B132" s="4" t="inlineStr">
@@ -4722,14 +4722,14 @@
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>SCM</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="D132" s="4" t="n"/>
       <c r="E132" s="4" t="n"/>
       <c r="F132" s="4" t="inlineStr">
         <is>
-          <t>1537</t>
+          <t>1515</t>
         </is>
       </c>
       <c r="G132" s="4" t="n"/>
@@ -4743,7 +4743,7 @@
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
         <is>
-          <t>Sunil Kumar</t>
+          <t>Radiologist 1</t>
         </is>
       </c>
       <c r="B133" s="4" t="inlineStr">
@@ -4753,14 +4753,14 @@
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>SCM</t>
+          <t>Radiologist 1</t>
         </is>
       </c>
       <c r="D133" s="4" t="n"/>
       <c r="E133" s="4" t="n"/>
       <c r="F133" s="4" t="inlineStr">
         <is>
-          <t>1538</t>
+          <t>1034</t>
         </is>
       </c>
       <c r="G133" s="4" t="n"/>
@@ -4774,7 +4774,7 @@
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
         <is>
-          <t>Vikas Kumar</t>
+          <t>Radiology reception</t>
         </is>
       </c>
       <c r="B134" s="4" t="inlineStr">
@@ -4784,14 +4784,14 @@
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>SCM</t>
+          <t>Radiology reception</t>
         </is>
       </c>
       <c r="D134" s="4" t="n"/>
       <c r="E134" s="4" t="n"/>
       <c r="F134" s="4" t="inlineStr">
         <is>
-          <t>1536</t>
+          <t>1030</t>
         </is>
       </c>
       <c r="G134" s="4" t="n"/>
@@ -4805,7 +4805,7 @@
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
         <is>
-          <t>Sample Receving</t>
+          <t>Radiology reception</t>
         </is>
       </c>
       <c r="B135" s="4" t="inlineStr">
@@ -4815,14 +4815,14 @@
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>Sample Receving</t>
+          <t>Radiology reception</t>
         </is>
       </c>
       <c r="D135" s="4" t="n"/>
       <c r="E135" s="4" t="n"/>
       <c r="F135" s="4" t="inlineStr">
         <is>
-          <t>1204</t>
+          <t>1031</t>
         </is>
       </c>
       <c r="G135" s="4" t="n"/>
@@ -4836,7 +4836,7 @@
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t>Deepak Vats</t>
+          <t>Registration Counter</t>
         </is>
       </c>
       <c r="B136" s="4" t="inlineStr">
@@ -4846,14 +4846,14 @@
       </c>
       <c r="C136" s="4" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Registration Counter</t>
         </is>
       </c>
       <c r="D136" s="4" t="n"/>
       <c r="E136" s="4" t="n"/>
       <c r="F136" s="4" t="inlineStr">
         <is>
-          <t>1598</t>
+          <t>1165</t>
         </is>
       </c>
       <c r="G136" s="4" t="n"/>
@@ -4867,7 +4867,7 @@
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
         <is>
-          <t>Services (Medical)</t>
+          <t>Registration Counter</t>
         </is>
       </c>
       <c r="B137" s="4" t="inlineStr">
@@ -4877,14 +4877,14 @@
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>Services (Medical)</t>
+          <t>Registration Counter</t>
         </is>
       </c>
       <c r="D137" s="4" t="n"/>
       <c r="E137" s="4" t="n"/>
       <c r="F137" s="4" t="inlineStr">
         <is>
-          <t>1250</t>
+          <t>1167</t>
         </is>
       </c>
       <c r="G137" s="4" t="n"/>
@@ -4898,7 +4898,7 @@
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
         <is>
-          <t>TMT</t>
+          <t>Registration Counter</t>
         </is>
       </c>
       <c r="B138" s="4" t="inlineStr">
@@ -4908,14 +4908,14 @@
       </c>
       <c r="C138" s="4" t="inlineStr">
         <is>
-          <t>TMT</t>
+          <t>Registration Counter</t>
         </is>
       </c>
       <c r="D138" s="4" t="n"/>
       <c r="E138" s="4" t="n"/>
       <c r="F138" s="4" t="inlineStr">
         <is>
-          <t>1072</t>
+          <t>1168</t>
         </is>
       </c>
       <c r="G138" s="4" t="n"/>
@@ -4929,7 +4929,7 @@
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>Registration Counter</t>
         </is>
       </c>
       <c r="B139" s="4" t="inlineStr">
@@ -4939,14 +4939,14 @@
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>Registration Counter</t>
         </is>
       </c>
       <c r="D139" s="4" t="n"/>
       <c r="E139" s="4" t="n"/>
       <c r="F139" s="4" t="inlineStr">
         <is>
-          <t>1063</t>
+          <t>1169</t>
         </is>
       </c>
       <c r="G139" s="4" t="n"/>
@@ -4960,7 +4960,7 @@
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>Adil</t>
         </is>
       </c>
       <c r="B140" s="4" t="inlineStr">
@@ -4970,14 +4970,14 @@
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>SCM</t>
         </is>
       </c>
       <c r="D140" s="4" t="n"/>
       <c r="E140" s="4" t="n"/>
       <c r="F140" s="4" t="inlineStr">
         <is>
-          <t>1064</t>
+          <t>1539</t>
         </is>
       </c>
       <c r="G140" s="4" t="n"/>
@@ -4991,7 +4991,7 @@
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
         <is>
-          <t>USG</t>
+          <t>Rajeev Kumar Malik</t>
         </is>
       </c>
       <c r="B141" s="4" t="inlineStr">
@@ -5001,14 +5001,14 @@
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>USG</t>
+          <t>SCM</t>
         </is>
       </c>
       <c r="D141" s="4" t="n"/>
       <c r="E141" s="4" t="n"/>
       <c r="F141" s="4" t="inlineStr">
         <is>
-          <t>1073</t>
+          <t>1537</t>
         </is>
       </c>
       <c r="G141" s="4" t="n"/>
@@ -5022,7 +5022,7 @@
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
         <is>
-          <t>USG Room 1</t>
+          <t>Sunil Kumar</t>
         </is>
       </c>
       <c r="B142" s="4" t="inlineStr">
@@ -5032,14 +5032,14 @@
       </c>
       <c r="C142" s="4" t="inlineStr">
         <is>
-          <t>USG Room 1</t>
+          <t>SCM</t>
         </is>
       </c>
       <c r="D142" s="4" t="n"/>
       <c r="E142" s="4" t="n"/>
       <c r="F142" s="4" t="inlineStr">
         <is>
-          <t>1036</t>
+          <t>1538</t>
         </is>
       </c>
       <c r="G142" s="4" t="n"/>
@@ -5053,7 +5053,7 @@
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t>Vinay- HR OPs</t>
+          <t>Vikas Kumar</t>
         </is>
       </c>
       <c r="B143" s="4" t="inlineStr">
@@ -5063,14 +5063,14 @@
       </c>
       <c r="C143" s="4" t="inlineStr">
         <is>
-          <t>Vinay- HR OPs</t>
+          <t>SCM</t>
         </is>
       </c>
       <c r="D143" s="4" t="n"/>
       <c r="E143" s="4" t="n"/>
       <c r="F143" s="4" t="inlineStr">
         <is>
-          <t>1578</t>
+          <t>1536</t>
         </is>
       </c>
       <c r="G143" s="4" t="n"/>
@@ -5081,8 +5081,287 @@
         </is>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" s="4" t="inlineStr">
+        <is>
+          <t>Sample Receving</t>
+        </is>
+      </c>
+      <c r="B144" s="4" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="C144" s="4" t="inlineStr">
+        <is>
+          <t>Sample Receving</t>
+        </is>
+      </c>
+      <c r="D144" s="4" t="n"/>
+      <c r="E144" s="4" t="n"/>
+      <c r="F144" s="4" t="inlineStr">
+        <is>
+          <t>1204</t>
+        </is>
+      </c>
+      <c r="G144" s="4" t="n"/>
+      <c r="H144" s="4" t="n"/>
+      <c r="I144" s="4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="4" t="inlineStr">
+        <is>
+          <t>Deepak Vats</t>
+        </is>
+      </c>
+      <c r="B145" s="4" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="C145" s="4" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="D145" s="4" t="n"/>
+      <c r="E145" s="4" t="n"/>
+      <c r="F145" s="4" t="inlineStr">
+        <is>
+          <t>1598</t>
+        </is>
+      </c>
+      <c r="G145" s="4" t="n"/>
+      <c r="H145" s="4" t="n"/>
+      <c r="I145" s="4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="4" t="inlineStr">
+        <is>
+          <t>Services (Medical)</t>
+        </is>
+      </c>
+      <c r="B146" s="4" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="C146" s="4" t="inlineStr">
+        <is>
+          <t>Services (Medical)</t>
+        </is>
+      </c>
+      <c r="D146" s="4" t="n"/>
+      <c r="E146" s="4" t="n"/>
+      <c r="F146" s="4" t="inlineStr">
+        <is>
+          <t>1250</t>
+        </is>
+      </c>
+      <c r="G146" s="4" t="n"/>
+      <c r="H146" s="4" t="n"/>
+      <c r="I146" s="4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="4" t="inlineStr">
+        <is>
+          <t>TMT</t>
+        </is>
+      </c>
+      <c r="B147" s="4" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="C147" s="4" t="inlineStr">
+        <is>
+          <t>TMT</t>
+        </is>
+      </c>
+      <c r="D147" s="4" t="n"/>
+      <c r="E147" s="4" t="n"/>
+      <c r="F147" s="4" t="inlineStr">
+        <is>
+          <t>1072</t>
+        </is>
+      </c>
+      <c r="G147" s="4" t="n"/>
+      <c r="H147" s="4" t="n"/>
+      <c r="I147" s="4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="4" t="inlineStr">
+        <is>
+          <t>TPA</t>
+        </is>
+      </c>
+      <c r="B148" s="4" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="C148" s="4" t="inlineStr">
+        <is>
+          <t>TPA</t>
+        </is>
+      </c>
+      <c r="D148" s="4" t="n"/>
+      <c r="E148" s="4" t="n"/>
+      <c r="F148" s="4" t="inlineStr">
+        <is>
+          <t>1063</t>
+        </is>
+      </c>
+      <c r="G148" s="4" t="n"/>
+      <c r="H148" s="4" t="n"/>
+      <c r="I148" s="4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="4" t="inlineStr">
+        <is>
+          <t>TPA</t>
+        </is>
+      </c>
+      <c r="B149" s="4" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="C149" s="4" t="inlineStr">
+        <is>
+          <t>TPA</t>
+        </is>
+      </c>
+      <c r="D149" s="4" t="n"/>
+      <c r="E149" s="4" t="n"/>
+      <c r="F149" s="4" t="inlineStr">
+        <is>
+          <t>1064</t>
+        </is>
+      </c>
+      <c r="G149" s="4" t="n"/>
+      <c r="H149" s="4" t="n"/>
+      <c r="I149" s="4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="4" t="inlineStr">
+        <is>
+          <t>USG</t>
+        </is>
+      </c>
+      <c r="B150" s="4" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="C150" s="4" t="inlineStr">
+        <is>
+          <t>USG</t>
+        </is>
+      </c>
+      <c r="D150" s="4" t="n"/>
+      <c r="E150" s="4" t="n"/>
+      <c r="F150" s="4" t="inlineStr">
+        <is>
+          <t>1073</t>
+        </is>
+      </c>
+      <c r="G150" s="4" t="n"/>
+      <c r="H150" s="4" t="n"/>
+      <c r="I150" s="4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="4" t="inlineStr">
+        <is>
+          <t>USG Room 1</t>
+        </is>
+      </c>
+      <c r="B151" s="4" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="C151" s="4" t="inlineStr">
+        <is>
+          <t>USG Room 1</t>
+        </is>
+      </c>
+      <c r="D151" s="4" t="n"/>
+      <c r="E151" s="4" t="n"/>
+      <c r="F151" s="4" t="inlineStr">
+        <is>
+          <t>1036</t>
+        </is>
+      </c>
+      <c r="G151" s="4" t="n"/>
+      <c r="H151" s="4" t="n"/>
+      <c r="I151" s="4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="4" t="inlineStr">
+        <is>
+          <t>Vinay OPs</t>
+        </is>
+      </c>
+      <c r="B152" s="4" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="C152" s="4" t="inlineStr">
+        <is>
+          <t>Vinay OPs</t>
+        </is>
+      </c>
+      <c r="D152" s="4" t="n"/>
+      <c r="E152" s="4" t="n"/>
+      <c r="F152" s="4" t="inlineStr">
+        <is>
+          <t>1578</t>
+        </is>
+      </c>
+      <c r="G152" s="4" t="n"/>
+      <c r="H152" s="4" t="n"/>
+      <c r="I152" s="4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I143"/>
+  <autoFilter ref="A1:I152"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>